<commit_message>
Fill required service params in feed (Consultations, WorkWithContract, Prepayment)
Avito rejected activation of all 30 restorable listings with error 1073:
these fields are required but empty in the official export. Default empty
cells to valid reference values so the next upload can activate them.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015QnZqbJyUMN7UW7q99jihd
</commit_message>
<xml_diff>
--- a/feed.xlsx
+++ b/feed.xlsx
@@ -1857,6 +1857,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA5" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -1967,6 +1982,16 @@
       <c r="V6" t="inlineStr">
         <is>
           <t>Удалённо</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -2269,6 +2294,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA8" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -2381,6 +2421,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y9" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -2498,6 +2548,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA10" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -2605,6 +2670,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA11" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -2715,6 +2795,16 @@
       <c r="V12" t="inlineStr">
         <is>
           <t>Удалённо</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -3127,6 +3217,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y15" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -3402,6 +3502,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y17" t="inlineStr">
         <is>
           <t>Нет</t>
@@ -3514,6 +3624,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA18" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -3626,6 +3751,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y19" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -3738,6 +3873,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA20" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -3845,6 +3995,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA21" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -3957,6 +4122,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA22" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4064,6 +4244,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA23" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4176,6 +4371,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA24" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4288,6 +4498,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y25" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -4405,6 +4625,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA26" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4517,6 +4752,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA27" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4624,6 +4874,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA28" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4731,6 +4996,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA29" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4838,6 +5118,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA30" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -4950,6 +5245,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA31" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -5057,6 +5367,16 @@
           <t>Есть</t>
         </is>
       </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="Z32" t="inlineStr">
         <is>
           <t>ИП | ООО | Другие юридические лица</t>
@@ -5169,6 +5489,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA33" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -5281,6 +5616,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA34" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -5398,6 +5748,11 @@
           <t>Есть</t>
         </is>
       </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y35" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -5515,6 +5870,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA36" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -5622,6 +5992,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y37" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -5744,6 +6124,11 @@
           <t>Да</t>
         </is>
       </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="Z38" t="inlineStr">
         <is>
           <t>ООО | Другие юридические лица</t>
@@ -5856,6 +6241,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA39" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -5958,6 +6358,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA40" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -6065,6 +6480,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA41" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -6177,6 +6607,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA42" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -6289,6 +6734,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y43" t="inlineStr">
         <is>
           <t>Нет</t>
@@ -6406,6 +6861,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA44" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -6508,6 +6978,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA45" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -6620,6 +7105,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA46" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -6874,6 +7374,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA48" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -6986,6 +7501,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA49" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -7098,6 +7628,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y50" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -7215,6 +7755,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA51" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -7327,6 +7882,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA52" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -7439,6 +8009,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA53" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -7551,6 +8136,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y54" t="inlineStr">
         <is>
           <t>Нет</t>
@@ -7663,6 +8258,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA55" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -7775,6 +8385,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA56" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -7887,6 +8512,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA57" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -7994,6 +8634,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA58" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -8248,6 +8903,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA60" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -8355,6 +9025,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA61" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -8457,6 +9142,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA62" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -8564,6 +9264,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y63" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -8676,6 +9386,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA64" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -8788,6 +9513,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA65" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -8895,6 +9635,16 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
       <c r="Y66" t="inlineStr">
         <is>
           <t>Нужна</t>
@@ -9007,6 +9757,21 @@
           <t>Удалённо</t>
         </is>
       </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="AA67" t="inlineStr">
         <is>
           <t>Понедельник | Вторник | Среда | Четверг | Пятница | Суббота | Воскресенье</t>
@@ -9117,6 +9882,21 @@
       <c r="V68" t="inlineStr">
         <is>
           <t>Удалённо</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Есть</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AA68" t="inlineStr">

</xml_diff>